<commit_message>
Add Competitive Index Table and Trends US2 regression suites.
Covers Improve Traffic CI views with POM specs, Excel workbooks, probes, npm scripts, and Allure HTML reports.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/BlueTriangle_Portal_Automation_Testing_Plan.xlsx
+++ b/docs/BlueTriangle_Portal_Automation_Testing_Plan.xlsx
@@ -1,16 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A1B3075-EC52-469A-B333-F3815CC723F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Summary" sheetId="1" r:id="rId1"/>
-    <sheet name="Automation Plan" sheetId="2" r:id="rId2"/>
-    <sheet name="Assumptions &amp; Notes" sheetId="3" r:id="rId3"/>
+    <sheet sheetId="1" name="Summary" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Automation Plan" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Assumptions &amp; Notes" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -22,7 +18,7 @@
     <t>Blue Triangle Portal — Comprehensive Automation Testing Plan</t>
   </si>
   <si>
-    <t>QA Automation — US2 (GDC Test Site 2)  |  Portal: https://portal.bluetriangle.com/  |  Plan as of 03-08-2026</t>
+    <t>QA Automation — US2 (GDC Test Site 2)  |  Portal: https://portal.bluetriangle.com/  |  Plan as of 03-Aug-2026</t>
   </si>
   <si>
     <t>Metric</t>
@@ -79,19 +75,19 @@
     <t>Plan start (completed work)</t>
   </si>
   <si>
-    <t>22-07-2026</t>
+    <t>22-Jul-2026</t>
   </si>
   <si>
     <t>Next screen start</t>
   </si>
   <si>
-    <t>04-08-2026</t>
+    <t>04-Aug-2026</t>
   </si>
   <si>
     <t>Projected plan end (incl. buffers)</t>
   </si>
   <si>
-    <t>17-11-2026</t>
+    <t>17-Nov-2026</t>
   </si>
   <si>
     <t>Profile / site focus</t>
@@ -208,49 +204,49 @@
     <t>Performance Detail</t>
   </si>
   <si>
-    <t>23-07-2026</t>
+    <t>23-Jul-2026</t>
   </si>
   <si>
     <t>Performance Comparison</t>
   </si>
   <si>
-    <t>24-07-2026</t>
+    <t>24-Jul-2026</t>
   </si>
   <si>
     <t>Aggregate Waterfall</t>
   </si>
   <si>
-    <t>25-07-2026</t>
+    <t>25-Jul-2026</t>
   </si>
   <si>
     <t>Bounce &amp; Exit Analysis</t>
   </si>
   <si>
-    <t>26-07-2026</t>
+    <t>26-Jul-2026</t>
   </si>
   <si>
     <t>Errors Explorer</t>
   </si>
   <si>
-    <t>27-07-2026</t>
+    <t>27-Jul-2026</t>
   </si>
   <si>
     <t>Performance Budget</t>
   </si>
   <si>
-    <t>28-07-2026</t>
+    <t>28-Jul-2026</t>
   </si>
   <si>
     <t>Session Lookup</t>
   </si>
   <si>
-    <t>29-07-2026</t>
+    <t>29-Jul-2026</t>
   </si>
   <si>
     <t>Revenue Opportunity</t>
   </si>
   <si>
-    <t>30-07-2026</t>
+    <t>30-Jul-2026</t>
   </si>
   <si>
     <t>First BI Improve Conversion screen completed.</t>
@@ -259,7 +255,7 @@
     <t>Marketing Overview</t>
   </si>
   <si>
-    <t>31-07-2026</t>
+    <t>31-Jul-2026</t>
   </si>
   <si>
     <t>Improve Traffic track started.</t>
@@ -268,7 +264,7 @@
     <t>Core Web Vitals (VitalScope)</t>
   </si>
   <si>
-    <t>01-08-2026</t>
+    <t>01-Aug-2026</t>
   </si>
   <si>
     <t>Same underlying RUM performance-overview route; covered via BI Improve Traffic path. RUM VitalScope leaf treated as same coverage.</t>
@@ -277,7 +273,7 @@
     <t>Customer Journey Analysis</t>
   </si>
   <si>
-    <t>02-08-2026</t>
+    <t>02-Aug-2026</t>
   </si>
   <si>
     <t>conversion-type=sales; Brand sibling is separate screen.</t>
@@ -286,7 +282,7 @@
     <t>Brand Customer Journey Analysis</t>
   </si>
   <si>
-    <t>03-08-2026</t>
+    <t>03-Aug-2026</t>
   </si>
   <si>
     <t>conversion-type=brand; completed 03-Aug-2026 (31/31 passed).</t>
@@ -307,7 +303,7 @@
     <t>Competitive Index Table</t>
   </si>
   <si>
-    <t>05-08-2026</t>
+    <t>05-Aug-2026</t>
   </si>
   <si>
     <t>view=table; pair with Trends screen.</t>
@@ -316,7 +312,7 @@
     <t>Competitive Index Trends</t>
   </si>
   <si>
-    <t>06-08-2026</t>
+    <t>06-Aug-2026</t>
   </si>
   <si>
     <t>view=trends; pair with Table screen.</t>
@@ -325,7 +321,7 @@
     <t>Bottom of the Sales Funnel Analysis</t>
   </si>
   <si>
-    <t>07-08-2026</t>
+    <t>07-Aug-2026</t>
   </si>
   <si>
     <t>Last Improve Traffic leaf in current catalog.</t>
@@ -334,10 +330,10 @@
     <t>[Buffer] Improve Traffic — bulk regression run &amp; failure fix</t>
   </si>
   <si>
-    <t>10-08-2026</t>
-  </si>
-  <si>
-    <t>11-08-2026</t>
+    <t>10-Aug-2026</t>
+  </si>
+  <si>
+    <t>11-Aug-2026</t>
   </si>
   <si>
     <t>Reserved after all screens in submodule (total 8: 4 already done + 4 newly scheduled). Run suites in bulk, triage flakes/hard failures, refresh Allure, update workbooks.</t>
@@ -346,7 +342,7 @@
     <t>Dashboards</t>
   </si>
   <si>
-    <t>12-08-2026</t>
+    <t>12-Aug-2026</t>
   </si>
   <si>
     <t>BI dashboards (exclude marketing=yes My Campaign).</t>
@@ -355,7 +351,7 @@
     <t>Revenue Analysis</t>
   </si>
   <si>
-    <t>13-08-2026</t>
+    <t>13-Aug-2026</t>
   </si>
   <si>
     <t>conversion-type=sales.</t>
@@ -364,7 +360,7 @@
     <t>Brand Opportunity</t>
   </si>
   <si>
-    <t>14-08-2026</t>
+    <t>14-Aug-2026</t>
   </si>
   <si>
     <t>Brand conversion sibling of Revenue Opportunity.</t>
@@ -373,7 +369,7 @@
     <t>Brand Analysis</t>
   </si>
   <si>
-    <t>17-08-2026</t>
+    <t>17-Aug-2026</t>
   </si>
   <si>
     <t>conversion-type=brand.</t>
@@ -382,19 +378,19 @@
     <t>Revenue Calculator</t>
   </si>
   <si>
-    <t>18-08-2026</t>
+    <t>18-Aug-2026</t>
   </si>
   <si>
     <t>Brand Calculator</t>
   </si>
   <si>
-    <t>19-08-2026</t>
+    <t>19-Aug-2026</t>
   </si>
   <si>
     <t>Revenue Attribution</t>
   </si>
   <si>
-    <t>20-08-2026</t>
+    <t>20-Aug-2026</t>
   </si>
   <si>
     <t>Read-only regression; do not mutate attribution config in automation.</t>
@@ -403,16 +399,16 @@
     <t>Brand Attribution</t>
   </si>
   <si>
-    <t>21-08-2026</t>
+    <t>21-Aug-2026</t>
   </si>
   <si>
     <t>[Buffer] Improve Conversion — bulk regression run &amp; failure fix</t>
   </si>
   <si>
-    <t>24-08-2026</t>
-  </si>
-  <si>
-    <t>25-08-2026</t>
+    <t>24-Aug-2026</t>
+  </si>
+  <si>
+    <t>25-Aug-2026</t>
   </si>
   <si>
     <t>Reserved after all screens in submodule (total 9: 1 already done + 8 newly scheduled). Run suites in bulk, triage flakes/hard failures, refresh Allure, update workbooks.</t>
@@ -421,7 +417,7 @@
     <t>Cart Refresh</t>
   </si>
   <si>
-    <t>26-08-2026</t>
+    <t>26-Aug-2026</t>
   </si>
   <si>
     <t>Broken-links / cart refresh analytics.</t>
@@ -430,7 +426,7 @@
     <t>Out of Stock</t>
   </si>
   <si>
-    <t>27-08-2026</t>
+    <t>27-Aug-2026</t>
   </si>
   <si>
     <t>Playwright regression (POM) + Allure + manual workbook.</t>
@@ -439,13 +435,13 @@
     <t>Revenue Assurance</t>
   </si>
   <si>
-    <t>28-08-2026</t>
+    <t>28-Aug-2026</t>
   </si>
   <si>
     <t>[Buffer] Improve Revenue — bulk regression run &amp; failure fix</t>
   </si>
   <si>
-    <t>31-08-2026</t>
+    <t>31-Aug-2026</t>
   </si>
   <si>
     <t>Reserved after all screens in submodule (total 3: 0 already done + 3 newly scheduled). Run suites in bulk, triage flakes/hard failures, refresh Allure, update workbooks.</t>
@@ -454,25 +450,25 @@
     <t>Digital Experience Overview</t>
   </si>
   <si>
-    <t>01-09-2026</t>
+    <t>01-Sep-2026</t>
   </si>
   <si>
     <t>Executive KPI Report</t>
   </si>
   <si>
-    <t>02-09-2026</t>
+    <t>02-Sep-2026</t>
   </si>
   <si>
     <t>CrUX Report</t>
   </si>
   <si>
-    <t>03-09-2026</t>
+    <t>03-Sep-2026</t>
   </si>
   <si>
     <t>Automated Reports</t>
   </si>
   <si>
-    <t>04-09-2026</t>
+    <t>04-Sep-2026</t>
   </si>
   <si>
     <t>List/view only — exclude create flows.</t>
@@ -481,13 +477,13 @@
     <t>Alerts</t>
   </si>
   <si>
-    <t>07-09-2026</t>
+    <t>07-Sep-2026</t>
   </si>
   <si>
     <t>Data Science</t>
   </si>
   <si>
-    <t>08-09-2026</t>
+    <t>08-Sep-2026</t>
   </si>
   <si>
     <t>Custom comparison / data science.</t>
@@ -496,7 +492,7 @@
     <t>[Buffer] Advanced Reporting &amp; Alerting — bulk regression run &amp; failure fix</t>
   </si>
   <si>
-    <t>09-09-2026</t>
+    <t>09-Sep-2026</t>
   </si>
   <si>
     <t>Reserved after all screens in submodule (total 6: 0 already done + 6 newly scheduled). Run suites in bulk, triage flakes/hard failures, refresh Allure, update workbooks.</t>
@@ -505,118 +501,118 @@
     <t>Alerts Log</t>
   </si>
   <si>
-    <t>10-09-2026</t>
+    <t>10-Sep-2026</t>
   </si>
   <si>
     <t>Reports Log</t>
   </si>
   <si>
-    <t>11-09-2026</t>
+    <t>11-Sep-2026</t>
   </si>
   <si>
     <t>Domain Violation &amp; Audit Log</t>
   </si>
   <si>
-    <t>14-09-2026</t>
+    <t>14-Sep-2026</t>
   </si>
   <si>
     <t>Synthetic Monitors Log</t>
   </si>
   <si>
-    <t>15-09-2026</t>
+    <t>15-Sep-2026</t>
   </si>
   <si>
     <t>Instant Measurement Log</t>
   </si>
   <si>
-    <t>16-09-2026</t>
+    <t>16-Sep-2026</t>
   </si>
   <si>
     <t>Consultant Access History</t>
   </si>
   <si>
-    <t>17-09-2026</t>
+    <t>17-Sep-2026</t>
   </si>
   <si>
     <t>Site Variables Log</t>
   </si>
   <si>
-    <t>18-09-2026</t>
+    <t>18-Sep-2026</t>
   </si>
   <si>
     <t>[Buffer] Logs — bulk regression run &amp; failure fix</t>
   </si>
   <si>
-    <t>21-09-2026</t>
-  </si>
-  <si>
-    <t>22-09-2026</t>
+    <t>21-Sep-2026</t>
+  </si>
+  <si>
+    <t>22-Sep-2026</t>
   </si>
   <si>
     <t>Reserved after all screens in submodule (total 7: 0 already done + 7 newly scheduled). Run suites in bulk, triage flakes/hard failures, refresh Allure, update workbooks.</t>
   </si>
   <si>
-    <t>23-09-2026</t>
+    <t>23-Sep-2026</t>
   </si>
   <si>
     <t>Native App overview (distinct from RUM Browser).</t>
   </si>
   <si>
-    <t>24-09-2026</t>
-  </si>
-  <si>
-    <t>25-09-2026</t>
-  </si>
-  <si>
-    <t>28-09-2026</t>
-  </si>
-  <si>
-    <t>29-09-2026</t>
+    <t>24-Sep-2026</t>
+  </si>
+  <si>
+    <t>25-Sep-2026</t>
+  </si>
+  <si>
+    <t>28-Sep-2026</t>
+  </si>
+  <si>
+    <t>29-Sep-2026</t>
   </si>
   <si>
     <t>[Buffer] Native App — bulk regression run &amp; failure fix</t>
   </si>
   <si>
-    <t>30-09-2026</t>
+    <t>30-Sep-2026</t>
   </si>
   <si>
     <t>Reserved after all screens in submodule (total 5: 0 already done + 5 newly scheduled). Run suites in bulk, triage flakes/hard failures, refresh Allure, update workbooks.</t>
   </si>
   <si>
-    <t>01-10-2026</t>
-  </si>
-  <si>
-    <t>02-10-2026</t>
+    <t>01-Oct-2026</t>
+  </si>
+  <si>
+    <t>02-Oct-2026</t>
   </si>
   <si>
     <t>Test Results</t>
   </si>
   <si>
-    <t>05-10-2026</t>
+    <t>05-Oct-2026</t>
   </si>
   <si>
     <t>Error State Tracking</t>
   </si>
   <si>
-    <t>06-10-2026</t>
+    <t>06-Oct-2026</t>
   </si>
   <si>
     <t>Page Performance Comparison</t>
   </si>
   <si>
-    <t>07-10-2026</t>
-  </si>
-  <si>
-    <t>08-10-2026</t>
-  </si>
-  <si>
-    <t>09-10-2026</t>
+    <t>07-Oct-2026</t>
+  </si>
+  <si>
+    <t>08-Oct-2026</t>
+  </si>
+  <si>
+    <t>09-Oct-2026</t>
   </si>
   <si>
     <t>Synthetic Monitors</t>
   </si>
   <si>
-    <t>12-10-2026</t>
+    <t>12-Oct-2026</t>
   </si>
   <si>
     <t>List/view — avoid create/edit/run write paths.</t>
@@ -625,124 +621,124 @@
     <t>Erroring Synthetic Monitors</t>
   </si>
   <si>
-    <t>13-10-2026</t>
+    <t>13-Oct-2026</t>
   </si>
   <si>
     <t>Synthetic Codes</t>
   </si>
   <si>
-    <t>14-10-2026</t>
+    <t>14-Oct-2026</t>
   </si>
   <si>
     <t>Central Data Repositories</t>
   </si>
   <si>
-    <t>15-10-2026</t>
+    <t>15-Oct-2026</t>
   </si>
   <si>
     <t>[Buffer] Synthetic — Real Browser — bulk regression run &amp; failure fix</t>
   </si>
   <si>
-    <t>16-10-2026</t>
-  </si>
-  <si>
-    <t>20-10-2026</t>
+    <t>16-Oct-2026</t>
+  </si>
+  <si>
+    <t>20-Oct-2026</t>
   </si>
   <si>
     <t>Reserved after all screens in submodule (total 11: 0 already done + 11 newly scheduled). Run suites in bulk, triage flakes/hard failures, refresh Allure, update workbooks.</t>
   </si>
   <si>
-    <t>21-10-2026</t>
+    <t>21-Oct-2026</t>
   </si>
   <si>
     <t>Base page overview.</t>
   </si>
   <si>
-    <t>22-10-2026</t>
+    <t>22-Oct-2026</t>
   </si>
   <si>
     <t>Base page &amp; SSL detail.</t>
   </si>
   <si>
-    <t>23-10-2026</t>
+    <t>23-Oct-2026</t>
   </si>
   <si>
     <t>[Buffer] Synthetic — API Checks (Base Page) — bulk regression run &amp; failure fix</t>
   </si>
   <si>
-    <t>26-10-2026</t>
-  </si>
-  <si>
-    <t>27-10-2026</t>
-  </si>
-  <si>
-    <t>28-10-2026</t>
-  </si>
-  <si>
-    <t>29-10-2026</t>
+    <t>26-Oct-2026</t>
+  </si>
+  <si>
+    <t>27-Oct-2026</t>
+  </si>
+  <si>
+    <t>28-Oct-2026</t>
+  </si>
+  <si>
+    <t>29-Oct-2026</t>
   </si>
   <si>
     <t>[Buffer] Network Health Checks — bulk regression run &amp; failure fix</t>
   </si>
   <si>
-    <t>30-10-2026</t>
+    <t>30-Oct-2026</t>
   </si>
   <si>
     <t>Tag &amp; Content Overview</t>
   </si>
   <si>
-    <t>02-11-2026</t>
+    <t>02-Nov-2026</t>
   </si>
   <si>
     <t>Domain Details</t>
   </si>
   <si>
-    <t>03-11-2026</t>
+    <t>03-Nov-2026</t>
   </si>
   <si>
     <t>Inventory Analysis</t>
   </si>
   <si>
-    <t>04-11-2026</t>
+    <t>04-Nov-2026</t>
   </si>
   <si>
     <t>Domain Baseline Analysis</t>
   </si>
   <si>
-    <t>05-11-2026</t>
+    <t>05-Nov-2026</t>
   </si>
   <si>
     <t>Service Profiles</t>
   </si>
   <si>
-    <t>06-11-2026</t>
+    <t>06-Nov-2026</t>
   </si>
   <si>
     <t>Service Details</t>
   </si>
   <si>
-    <t>09-11-2026</t>
+    <t>09-Nov-2026</t>
   </si>
   <si>
     <t>SLA Status</t>
   </si>
   <si>
-    <t>10-11-2026</t>
+    <t>10-Nov-2026</t>
   </si>
   <si>
     <t>[Buffer] CSP &amp; Tag Governance — bulk regression run &amp; failure fix</t>
   </si>
   <si>
-    <t>11-11-2026</t>
-  </si>
-  <si>
-    <t>12-11-2026</t>
+    <t>11-Nov-2026</t>
+  </si>
+  <si>
+    <t>12-Nov-2026</t>
   </si>
   <si>
     <t>My Account</t>
   </si>
   <si>
-    <t>13-11-2026</t>
+    <t>13-Nov-2026</t>
   </si>
   <si>
     <t>View-only profile/account settings.</t>
@@ -751,7 +747,7 @@
     <t>View Profile</t>
   </si>
   <si>
-    <t>16-11-2026</t>
+    <t>16-Nov-2026</t>
   </si>
   <si>
     <t>View-only.</t>
@@ -856,114 +852,91 @@
     <t>• Plan should be re-baselined if portal menu adds/removes leaves or if capacity changes (multiple engineers).</t>
   </si>
   <si>
-    <t>Generated: 03-08-2026  |  Regenerate: node scripts/generate-portal-automation-plan.js</t>
+    <t>Generated: 03-Aug-2026  |  Regenerate: node scripts/generate-portal-automation-plan.js</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="17" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="16"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="10"/>
-      <color rgb="FF595959"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FF595959"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b/>
+    </font>
+    <font>
+      <b/>
       <color rgb="FF006100"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
       <color rgb="FF1F4E79"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
       <color rgb="FFC65911"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
       <color rgb="FF9C5700"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
       <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FF006100"/>
       <sz val="10"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <i/>
-      <sz val="11"/>
       <color rgb="FFC65911"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FF1F4E79"/>
       <sz val="10"/>
-      <color rgb="FF1F4E79"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFC65911"/>
       <sz val="10"/>
-      <color rgb="FFC65911"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FF0D2B4A"/>
       <sz val="14"/>
-      <color rgb="FF0D2B4A"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FF1F4E79"/>
       <sz val="12"/>
-      <color rgb="FF1F4E79"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="13">
@@ -1043,6 +1016,10 @@
   </cellStyleXfs>
   <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1098,10 +1075,6 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1440,179 +1413,179 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E43"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
-    <col min="2" max="2" width="50.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+    <row r="1" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-    </row>
-    <row r="4" spans="1:4" s="1" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="4" ht="28" customHeight="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B5">
         <v>72</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
         <v>5</v>
       </c>
       <c r="B6">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
         <v>6</v>
       </c>
       <c r="B7">
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>7</v>
       </c>
       <c r="B8">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="4" t="s">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B10">
         <v>712</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B11">
         <v>120</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
         <v>12</v>
       </c>
       <c r="B12">
         <v>592</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
         <v>13</v>
       </c>
       <c r="B13" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
         <v>15</v>
       </c>
       <c r="B14" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
         <v>17</v>
       </c>
       <c r="B15" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
         <v>19</v>
       </c>
       <c r="B16" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
         <v>21</v>
       </c>
       <c r="B17" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
         <v>23</v>
       </c>
       <c r="B18" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
         <v>25</v>
       </c>
       <c r="B19" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="5" t="s">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="7" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:5" s="1" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
+    <row r="23" ht="28" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D23" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="E23" s="3" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1623,7 +1596,7 @@
       <c r="B24" t="s">
         <v>34</v>
       </c>
-      <c r="C24" s="6">
+      <c r="C24" s="8">
         <v>8</v>
       </c>
       <c r="D24">
@@ -1640,7 +1613,7 @@
       <c r="B25" t="s">
         <v>36</v>
       </c>
-      <c r="C25" s="7">
+      <c r="C25" s="9">
         <v>1</v>
       </c>
       <c r="D25">
@@ -1657,7 +1630,7 @@
       <c r="B26" t="s">
         <v>37</v>
       </c>
-      <c r="C26" s="7">
+      <c r="C26" s="9">
         <v>4</v>
       </c>
       <c r="D26">
@@ -1820,33 +1793,33 @@
         <v>4</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="8" t="s">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" s="10" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="4" t="s">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="9" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="10" t="s">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" s="12" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="11" t="s">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" s="13" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="12" t="s">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" s="14" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1856,14 +1829,14 @@
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I85"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -1875,2493 +1848,2496 @@
     <col min="9" max="9" width="62" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="3" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="14">
+    <row r="2" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="16">
         <v>1</v>
       </c>
-      <c r="B2" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="C2" s="15" t="s">
+      <c r="B2" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="E2" s="14">
-        <v>8</v>
-      </c>
-      <c r="F2" s="14" t="s">
+      <c r="E2" s="16">
+        <v>8</v>
+      </c>
+      <c r="F2" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="G2" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="16" t="s">
+      <c r="H2" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="I2" s="13" t="s">
+      <c r="I2" s="15" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="14">
+    <row r="3" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="16">
         <v>2</v>
       </c>
-      <c r="B3" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="C3" s="15" t="s">
+      <c r="B3" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="E3" s="14">
-        <v>8</v>
-      </c>
-      <c r="F3" s="14" t="s">
+      <c r="E3" s="16">
+        <v>8</v>
+      </c>
+      <c r="F3" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="G3" s="14" t="s">
+      <c r="G3" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="H3" s="16" t="s">
+      <c r="H3" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="I3" s="13" t="s">
+      <c r="I3" s="15" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="14">
+    <row r="4" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="16">
         <v>3</v>
       </c>
-      <c r="B4" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="C4" s="15" t="s">
+      <c r="B4" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="E4" s="14">
-        <v>8</v>
-      </c>
-      <c r="F4" s="14" t="s">
+      <c r="E4" s="16">
+        <v>8</v>
+      </c>
+      <c r="F4" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="G4" s="14" t="s">
+      <c r="G4" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="H4" s="16" t="s">
+      <c r="H4" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="13" t="s">
+      <c r="I4" s="15" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="14">
+    <row r="5" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="16">
         <v>4</v>
       </c>
-      <c r="B5" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="C5" s="15" t="s">
+      <c r="B5" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="E5" s="14">
-        <v>8</v>
-      </c>
-      <c r="F5" s="14" t="s">
+      <c r="E5" s="16">
+        <v>8</v>
+      </c>
+      <c r="F5" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="G5" s="14" t="s">
+      <c r="G5" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="H5" s="16" t="s">
+      <c r="H5" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="I5" s="13" t="s">
+      <c r="I5" s="15" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="6" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="14">
+    <row r="6" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="16">
         <v>5</v>
       </c>
-      <c r="B6" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" s="15" t="s">
+      <c r="B6" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="15" t="s">
+      <c r="D6" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="E6" s="14">
-        <v>8</v>
-      </c>
-      <c r="F6" s="14" t="s">
+      <c r="E6" s="16">
+        <v>8</v>
+      </c>
+      <c r="F6" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="G6" s="14" t="s">
+      <c r="G6" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="H6" s="16" t="s">
+      <c r="H6" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="I6" s="13" t="s">
+      <c r="I6" s="15" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="7" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="14">
+    <row r="7" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="16">
         <v>6</v>
       </c>
-      <c r="B7" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="C7" s="15" t="s">
+      <c r="B7" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="D7" s="15" t="s">
+      <c r="D7" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="E7" s="14">
-        <v>8</v>
-      </c>
-      <c r="F7" s="14" t="s">
+      <c r="E7" s="16">
+        <v>8</v>
+      </c>
+      <c r="F7" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="G7" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="H7" s="16" t="s">
+      <c r="H7" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="I7" s="13" t="s">
+      <c r="I7" s="15" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="8" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="14">
+    <row r="8" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="16">
         <v>7</v>
       </c>
-      <c r="B8" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="C8" s="15" t="s">
+      <c r="B8" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="15" t="s">
+      <c r="D8" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="E8" s="14">
-        <v>8</v>
-      </c>
-      <c r="F8" s="14" t="s">
+      <c r="E8" s="16">
+        <v>8</v>
+      </c>
+      <c r="F8" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="G8" s="14" t="s">
+      <c r="G8" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="H8" s="16" t="s">
+      <c r="H8" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="I8" s="13" t="s">
+      <c r="I8" s="15" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="14">
-        <v>8</v>
-      </c>
-      <c r="B9" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="C9" s="15" t="s">
+    <row r="9" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="16">
+        <v>8</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="15" t="s">
+      <c r="D9" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="E9" s="14">
-        <v>8</v>
-      </c>
-      <c r="F9" s="14" t="s">
+      <c r="E9" s="16">
+        <v>8</v>
+      </c>
+      <c r="F9" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="G9" s="14" t="s">
+      <c r="G9" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="H9" s="16" t="s">
+      <c r="H9" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="I9" s="13" t="s">
+      <c r="I9" s="15" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="14">
+    <row r="10" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="16">
         <v>9</v>
       </c>
-      <c r="B10" s="15" t="s">
+      <c r="B10" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="E10" s="14">
-        <v>8</v>
-      </c>
-      <c r="F10" s="14" t="s">
+      <c r="E10" s="16">
+        <v>8</v>
+      </c>
+      <c r="F10" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="G10" s="14" t="s">
+      <c r="G10" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="H10" s="16" t="s">
+      <c r="H10" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="I10" s="13" t="s">
+      <c r="I10" s="15" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="11" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="14">
+    <row r="11" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="16">
         <v>10</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="D11" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="E11" s="14">
-        <v>8</v>
-      </c>
-      <c r="F11" s="14" t="s">
+      <c r="E11" s="16">
+        <v>8</v>
+      </c>
+      <c r="F11" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="G11" s="14" t="s">
+      <c r="G11" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="H11" s="16" t="s">
+      <c r="H11" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="I11" s="13" t="s">
+      <c r="I11" s="15" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="12" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="14">
+    <row r="12" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="16">
         <v>11</v>
       </c>
-      <c r="B12" s="15" t="s">
+      <c r="B12" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="C12" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="D12" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="E12" s="14">
-        <v>8</v>
-      </c>
-      <c r="F12" s="14" t="s">
+      <c r="E12" s="16">
+        <v>8</v>
+      </c>
+      <c r="F12" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="G12" s="14" t="s">
+      <c r="G12" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="H12" s="16" t="s">
+      <c r="H12" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="I12" s="13" t="s">
+      <c r="I12" s="15" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="13" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="14">
+    <row r="13" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="16">
         <v>12</v>
       </c>
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="15" t="s">
+      <c r="C13" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="D13" s="15" t="s">
+      <c r="D13" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="E13" s="14">
-        <v>8</v>
-      </c>
-      <c r="F13" s="14" t="s">
+      <c r="E13" s="16">
+        <v>8</v>
+      </c>
+      <c r="F13" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="G13" s="14" t="s">
+      <c r="G13" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="H13" s="16" t="s">
+      <c r="H13" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="I13" s="13" t="s">
+      <c r="I13" s="15" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="14">
+    <row r="14" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="16">
         <v>13</v>
       </c>
-      <c r="B14" s="15" t="s">
+      <c r="B14" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="C14" s="15" t="s">
+      <c r="C14" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="D14" s="15" t="s">
+      <c r="D14" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="E14" s="14">
-        <v>8</v>
-      </c>
-      <c r="F14" s="14" t="s">
+      <c r="E14" s="16">
+        <v>8</v>
+      </c>
+      <c r="F14" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="G14" s="14" t="s">
+      <c r="G14" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="H14" s="16" t="s">
+      <c r="H14" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="I14" s="13" t="s">
+      <c r="I14" s="15" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="15" spans="1:9" s="13" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="17">
+    <row r="15" ht="36" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="19">
         <v>14</v>
       </c>
-      <c r="B15" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="C15" s="18" t="s">
+      <c r="B15" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="D15" s="19" t="s">
+      <c r="D15" s="21" t="s">
         <v>91</v>
       </c>
-      <c r="E15" s="17">
+      <c r="E15" s="19">
         <v>16</v>
       </c>
-      <c r="F15" s="17" t="s">
+      <c r="F15" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="G15" s="17" t="s">
+      <c r="G15" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="H15" s="16" t="s">
+      <c r="H15" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="I15" s="13" t="s">
+      <c r="I15" s="15" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="16" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="20">
+    <row r="16" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="22">
         <v>15</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="B16" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="C16" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="D16" s="13" t="s">
+      <c r="D16" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="E16" s="20">
-        <v>8</v>
-      </c>
-      <c r="F16" s="20" t="s">
+      <c r="E16" s="22">
+        <v>8</v>
+      </c>
+      <c r="F16" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="G16" s="20" t="s">
+      <c r="G16" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="H16" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I16" s="13" t="s">
+      <c r="H16" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I16" s="15" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="17" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="22">
+    <row r="17" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="24">
         <v>16</v>
       </c>
-      <c r="B17" s="23" t="s">
+      <c r="B17" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="C17" s="23" t="s">
+      <c r="C17" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="D17" s="23" t="s">
+      <c r="D17" s="25" t="s">
         <v>95</v>
       </c>
-      <c r="E17" s="22">
-        <v>8</v>
-      </c>
-      <c r="F17" s="22" t="s">
+      <c r="E17" s="24">
+        <v>8</v>
+      </c>
+      <c r="F17" s="24" t="s">
         <v>96</v>
       </c>
-      <c r="G17" s="22" t="s">
+      <c r="G17" s="24" t="s">
         <v>96</v>
       </c>
-      <c r="H17" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I17" s="13" t="s">
+      <c r="H17" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I17" s="15" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="18" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="20">
+    <row r="18" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="22">
         <v>17</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="D18" s="13" t="s">
+      <c r="D18" s="15" t="s">
         <v>98</v>
       </c>
-      <c r="E18" s="20">
-        <v>8</v>
-      </c>
-      <c r="F18" s="20" t="s">
+      <c r="E18" s="22">
+        <v>8</v>
+      </c>
+      <c r="F18" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="G18" s="20" t="s">
+      <c r="G18" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="H18" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I18" s="13" t="s">
+      <c r="H18" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I18" s="15" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="19" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="22">
+    <row r="19" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="24">
         <v>18</v>
       </c>
-      <c r="B19" s="23" t="s">
+      <c r="B19" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="C19" s="23" t="s">
+      <c r="C19" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="D19" s="23" t="s">
+      <c r="D19" s="25" t="s">
         <v>101</v>
       </c>
-      <c r="E19" s="22">
-        <v>8</v>
-      </c>
-      <c r="F19" s="22" t="s">
+      <c r="E19" s="24">
+        <v>8</v>
+      </c>
+      <c r="F19" s="24" t="s">
         <v>102</v>
       </c>
-      <c r="G19" s="22" t="s">
+      <c r="G19" s="24" t="s">
         <v>102</v>
       </c>
-      <c r="H19" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I19" s="13" t="s">
+      <c r="H19" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I19" s="15" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="20" spans="1:9" s="13" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="17">
+    <row r="20" ht="36" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="19">
         <v>19</v>
       </c>
-      <c r="B20" s="18" t="s">
+      <c r="B20" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="C20" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="D20" s="19" t="s">
+      <c r="D20" s="21" t="s">
         <v>104</v>
       </c>
-      <c r="E20" s="17">
+      <c r="E20" s="19">
         <v>16</v>
       </c>
-      <c r="F20" s="17" t="s">
+      <c r="F20" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="G20" s="17" t="s">
+      <c r="G20" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="H20" s="24" t="s">
+      <c r="H20" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="I20" s="13" t="s">
+      <c r="I20" s="15" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="21" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="22">
+    <row r="21" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="24">
         <v>20</v>
       </c>
-      <c r="B21" s="23" t="s">
+      <c r="B21" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="23" t="s">
+      <c r="C21" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="D21" s="23" t="s">
+      <c r="D21" s="25" t="s">
         <v>108</v>
       </c>
-      <c r="E21" s="22">
-        <v>8</v>
-      </c>
-      <c r="F21" s="22" t="s">
+      <c r="E21" s="24">
+        <v>8</v>
+      </c>
+      <c r="F21" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="G21" s="22" t="s">
+      <c r="G21" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="H21" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I21" s="13" t="s">
+      <c r="H21" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I21" s="15" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="22" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="20">
+    <row r="22" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="22">
         <v>21</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="C22" s="13" t="s">
+      <c r="C22" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="D22" s="13" t="s">
+      <c r="D22" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="E22" s="20">
-        <v>8</v>
-      </c>
-      <c r="F22" s="20" t="s">
+      <c r="E22" s="22">
+        <v>8</v>
+      </c>
+      <c r="F22" s="22" t="s">
         <v>112</v>
       </c>
-      <c r="G22" s="20" t="s">
+      <c r="G22" s="22" t="s">
         <v>112</v>
       </c>
-      <c r="H22" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I22" s="13" t="s">
+      <c r="H22" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I22" s="15" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="23" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="22">
+    <row r="23" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="24">
         <v>22</v>
       </c>
-      <c r="B23" s="23" t="s">
+      <c r="B23" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="C23" s="23" t="s">
+      <c r="C23" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="D23" s="23" t="s">
+      <c r="D23" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="E23" s="22">
-        <v>8</v>
-      </c>
-      <c r="F23" s="22" t="s">
+      <c r="E23" s="24">
+        <v>8</v>
+      </c>
+      <c r="F23" s="24" t="s">
         <v>115</v>
       </c>
-      <c r="G23" s="22" t="s">
+      <c r="G23" s="24" t="s">
         <v>115</v>
       </c>
-      <c r="H23" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I23" s="13" t="s">
+      <c r="H23" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I23" s="15" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="24" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="20">
+    <row r="24" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="22">
         <v>23</v>
       </c>
-      <c r="B24" s="13" t="s">
+      <c r="B24" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="C24" s="13" t="s">
+      <c r="C24" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="D24" s="13" t="s">
+      <c r="D24" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="E24" s="20">
-        <v>8</v>
-      </c>
-      <c r="F24" s="20" t="s">
+      <c r="E24" s="22">
+        <v>8</v>
+      </c>
+      <c r="F24" s="22" t="s">
         <v>118</v>
       </c>
-      <c r="G24" s="20" t="s">
+      <c r="G24" s="22" t="s">
         <v>118</v>
       </c>
-      <c r="H24" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I24" s="13" t="s">
+      <c r="H24" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I24" s="15" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="25" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="22">
+    <row r="25" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="24">
         <v>24</v>
       </c>
-      <c r="B25" s="23" t="s">
+      <c r="B25" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="C25" s="23" t="s">
+      <c r="C25" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="D25" s="23" t="s">
+      <c r="D25" s="25" t="s">
         <v>120</v>
       </c>
-      <c r="E25" s="22">
-        <v>8</v>
-      </c>
-      <c r="F25" s="22" t="s">
+      <c r="E25" s="24">
+        <v>8</v>
+      </c>
+      <c r="F25" s="24" t="s">
         <v>121</v>
       </c>
-      <c r="G25" s="22" t="s">
+      <c r="G25" s="24" t="s">
         <v>121</v>
       </c>
-      <c r="H25" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I25" s="13" t="s">
+      <c r="H25" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I25" s="15" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="26" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="20">
+    <row r="26" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="22">
         <v>25</v>
       </c>
-      <c r="B26" s="13" t="s">
+      <c r="B26" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="C26" s="13" t="s">
+      <c r="C26" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="D26" s="13" t="s">
+      <c r="D26" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="E26" s="20">
-        <v>8</v>
-      </c>
-      <c r="F26" s="20" t="s">
+      <c r="E26" s="22">
+        <v>8</v>
+      </c>
+      <c r="F26" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="G26" s="20" t="s">
+      <c r="G26" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="H26" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I26" s="13" t="s">
+      <c r="H26" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I26" s="15" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="27" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="22">
+    <row r="27" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="24">
         <v>26</v>
       </c>
-      <c r="B27" s="23" t="s">
+      <c r="B27" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="C27" s="23" t="s">
+      <c r="C27" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="D27" s="23" t="s">
+      <c r="D27" s="25" t="s">
         <v>124</v>
       </c>
-      <c r="E27" s="22">
-        <v>8</v>
-      </c>
-      <c r="F27" s="22" t="s">
+      <c r="E27" s="24">
+        <v>8</v>
+      </c>
+      <c r="F27" s="24" t="s">
         <v>125</v>
       </c>
-      <c r="G27" s="22" t="s">
+      <c r="G27" s="24" t="s">
         <v>125</v>
       </c>
-      <c r="H27" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I27" s="13" t="s">
+      <c r="H27" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I27" s="15" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="28" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="20">
+    <row r="28" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="22">
         <v>27</v>
       </c>
-      <c r="B28" s="13" t="s">
+      <c r="B28" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="C28" s="13" t="s">
+      <c r="C28" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="D28" s="13" t="s">
+      <c r="D28" s="15" t="s">
         <v>127</v>
       </c>
-      <c r="E28" s="20">
-        <v>8</v>
-      </c>
-      <c r="F28" s="20" t="s">
+      <c r="E28" s="22">
+        <v>8</v>
+      </c>
+      <c r="F28" s="22" t="s">
         <v>128</v>
       </c>
-      <c r="G28" s="20" t="s">
+      <c r="G28" s="22" t="s">
         <v>128</v>
       </c>
-      <c r="H28" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I28" s="13" t="s">
+      <c r="H28" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I28" s="15" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="29" spans="1:9" s="13" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="17">
+    <row r="29" ht="36" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="19">
         <v>28</v>
       </c>
-      <c r="B29" s="18" t="s">
+      <c r="B29" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="C29" s="18" t="s">
+      <c r="C29" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="D29" s="19" t="s">
+      <c r="D29" s="21" t="s">
         <v>129</v>
       </c>
-      <c r="E29" s="17">
+      <c r="E29" s="19">
         <v>16</v>
       </c>
-      <c r="F29" s="17" t="s">
+      <c r="F29" s="19" t="s">
         <v>130</v>
       </c>
-      <c r="G29" s="17" t="s">
+      <c r="G29" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="H29" s="24" t="s">
+      <c r="H29" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="I29" s="13" t="s">
+      <c r="I29" s="15" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="30" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="20">
+    <row r="30" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="22">
         <v>29</v>
       </c>
-      <c r="B30" s="13" t="s">
+      <c r="B30" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="C30" s="13" t="s">
+      <c r="C30" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="D30" s="13" t="s">
+      <c r="D30" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="E30" s="20">
-        <v>8</v>
-      </c>
-      <c r="F30" s="20" t="s">
+      <c r="E30" s="22">
+        <v>8</v>
+      </c>
+      <c r="F30" s="22" t="s">
         <v>134</v>
       </c>
-      <c r="G30" s="20" t="s">
+      <c r="G30" s="22" t="s">
         <v>134</v>
       </c>
-      <c r="H30" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I30" s="13" t="s">
+      <c r="H30" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I30" s="15" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="31" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="22">
+    <row r="31" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="24">
         <v>30</v>
       </c>
-      <c r="B31" s="23" t="s">
+      <c r="B31" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="C31" s="23" t="s">
+      <c r="C31" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="D31" s="23" t="s">
+      <c r="D31" s="25" t="s">
         <v>136</v>
       </c>
-      <c r="E31" s="22">
-        <v>8</v>
-      </c>
-      <c r="F31" s="22" t="s">
+      <c r="E31" s="24">
+        <v>8</v>
+      </c>
+      <c r="F31" s="24" t="s">
         <v>137</v>
       </c>
-      <c r="G31" s="22" t="s">
+      <c r="G31" s="24" t="s">
         <v>137</v>
       </c>
-      <c r="H31" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I31" s="13" t="s">
+      <c r="H31" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I31" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="32" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="20">
+    <row r="32" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="22">
         <v>31</v>
       </c>
-      <c r="B32" s="13" t="s">
+      <c r="B32" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="C32" s="13" t="s">
+      <c r="C32" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="D32" s="13" t="s">
+      <c r="D32" s="15" t="s">
         <v>139</v>
       </c>
-      <c r="E32" s="20">
-        <v>8</v>
-      </c>
-      <c r="F32" s="20" t="s">
+      <c r="E32" s="22">
+        <v>8</v>
+      </c>
+      <c r="F32" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="G32" s="20" t="s">
+      <c r="G32" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="H32" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I32" s="13" t="s">
+      <c r="H32" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I32" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="33" spans="1:9" s="13" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="17">
+    <row r="33" ht="36" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="19">
         <v>32</v>
       </c>
-      <c r="B33" s="18" t="s">
+      <c r="B33" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="C33" s="18" t="s">
+      <c r="C33" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="D33" s="19" t="s">
+      <c r="D33" s="21" t="s">
         <v>141</v>
       </c>
-      <c r="E33" s="17">
+      <c r="E33" s="19">
         <v>4</v>
       </c>
-      <c r="F33" s="17" t="s">
+      <c r="F33" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="G33" s="17" t="s">
+      <c r="G33" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="H33" s="24" t="s">
+      <c r="H33" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="I33" s="13" t="s">
+      <c r="I33" s="15" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="34" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="20">
-        <v>33</v>
-      </c>
-      <c r="B34" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C34" s="13" t="s">
+    <row r="34" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="22">
+        <v>33</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C34" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="D34" s="13" t="s">
+      <c r="D34" s="15" t="s">
         <v>144</v>
       </c>
-      <c r="E34" s="20">
-        <v>8</v>
-      </c>
-      <c r="F34" s="20" t="s">
+      <c r="E34" s="22">
+        <v>8</v>
+      </c>
+      <c r="F34" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="G34" s="20" t="s">
+      <c r="G34" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="H34" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I34" s="13" t="s">
+      <c r="H34" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I34" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="35" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="22">
+    <row r="35" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="24">
         <v>34</v>
       </c>
-      <c r="B35" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C35" s="23" t="s">
+      <c r="B35" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C35" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="D35" s="23" t="s">
+      <c r="D35" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="E35" s="22">
-        <v>8</v>
-      </c>
-      <c r="F35" s="22" t="s">
+      <c r="E35" s="24">
+        <v>8</v>
+      </c>
+      <c r="F35" s="24" t="s">
         <v>147</v>
       </c>
-      <c r="G35" s="22" t="s">
+      <c r="G35" s="24" t="s">
         <v>147</v>
       </c>
-      <c r="H35" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I35" s="13" t="s">
+      <c r="H35" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I35" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="36" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="20">
+    <row r="36" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="22">
         <v>35</v>
       </c>
-      <c r="B36" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C36" s="13" t="s">
+      <c r="B36" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C36" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="D36" s="13" t="s">
+      <c r="D36" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="E36" s="20">
-        <v>8</v>
-      </c>
-      <c r="F36" s="20" t="s">
+      <c r="E36" s="22">
+        <v>8</v>
+      </c>
+      <c r="F36" s="22" t="s">
         <v>149</v>
       </c>
-      <c r="G36" s="20" t="s">
+      <c r="G36" s="22" t="s">
         <v>149</v>
       </c>
-      <c r="H36" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I36" s="13" t="s">
+      <c r="H36" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I36" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="37" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="22">
+    <row r="37" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="24">
         <v>36</v>
       </c>
-      <c r="B37" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C37" s="23" t="s">
+      <c r="B37" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C37" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="D37" s="23" t="s">
+      <c r="D37" s="25" t="s">
         <v>150</v>
       </c>
-      <c r="E37" s="22">
-        <v>8</v>
-      </c>
-      <c r="F37" s="22" t="s">
+      <c r="E37" s="24">
+        <v>8</v>
+      </c>
+      <c r="F37" s="24" t="s">
         <v>151</v>
       </c>
-      <c r="G37" s="22" t="s">
+      <c r="G37" s="24" t="s">
         <v>151</v>
       </c>
-      <c r="H37" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I37" s="13" t="s">
+      <c r="H37" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I37" s="15" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="38" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="20">
+    <row r="38" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="22">
         <v>37</v>
       </c>
-      <c r="B38" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C38" s="13" t="s">
+      <c r="B38" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C38" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="D38" s="13" t="s">
+      <c r="D38" s="15" t="s">
         <v>153</v>
       </c>
-      <c r="E38" s="20">
-        <v>8</v>
-      </c>
-      <c r="F38" s="20" t="s">
+      <c r="E38" s="22">
+        <v>8</v>
+      </c>
+      <c r="F38" s="22" t="s">
         <v>154</v>
       </c>
-      <c r="G38" s="20" t="s">
+      <c r="G38" s="22" t="s">
         <v>154</v>
       </c>
-      <c r="H38" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I38" s="13" t="s">
+      <c r="H38" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I38" s="15" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="39" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="22">
+    <row r="39" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="24">
         <v>38</v>
       </c>
-      <c r="B39" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C39" s="23" t="s">
+      <c r="B39" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C39" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="D39" s="23" t="s">
+      <c r="D39" s="25" t="s">
         <v>155</v>
       </c>
-      <c r="E39" s="22">
-        <v>8</v>
-      </c>
-      <c r="F39" s="22" t="s">
+      <c r="E39" s="24">
+        <v>8</v>
+      </c>
+      <c r="F39" s="24" t="s">
         <v>156</v>
       </c>
-      <c r="G39" s="22" t="s">
+      <c r="G39" s="24" t="s">
         <v>156</v>
       </c>
-      <c r="H39" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I39" s="13" t="s">
+      <c r="H39" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I39" s="15" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="40" spans="1:9" s="13" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="17">
+    <row r="40" ht="36" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="19">
         <v>39</v>
       </c>
-      <c r="B40" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="C40" s="18" t="s">
+      <c r="B40" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="C40" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="D40" s="19" t="s">
+      <c r="D40" s="21" t="s">
         <v>158</v>
       </c>
-      <c r="E40" s="17">
-        <v>8</v>
-      </c>
-      <c r="F40" s="17" t="s">
+      <c r="E40" s="19">
+        <v>8</v>
+      </c>
+      <c r="F40" s="19" t="s">
         <v>159</v>
       </c>
-      <c r="G40" s="17" t="s">
+      <c r="G40" s="19" t="s">
         <v>159</v>
       </c>
-      <c r="H40" s="24" t="s">
+      <c r="H40" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="I40" s="13" t="s">
+      <c r="I40" s="15" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="41" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="22">
+    <row r="41" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="24">
         <v>40</v>
       </c>
-      <c r="B41" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C41" s="23" t="s">
+      <c r="B41" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C41" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="D41" s="23" t="s">
+      <c r="D41" s="25" t="s">
         <v>161</v>
       </c>
-      <c r="E41" s="22">
-        <v>8</v>
-      </c>
-      <c r="F41" s="22" t="s">
+      <c r="E41" s="24">
+        <v>8</v>
+      </c>
+      <c r="F41" s="24" t="s">
         <v>162</v>
       </c>
-      <c r="G41" s="22" t="s">
+      <c r="G41" s="24" t="s">
         <v>162</v>
       </c>
-      <c r="H41" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I41" s="13" t="s">
+      <c r="H41" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I41" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="42" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="20">
+    <row r="42" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="22">
         <v>41</v>
       </c>
-      <c r="B42" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C42" s="13" t="s">
+      <c r="B42" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C42" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="D42" s="13" t="s">
+      <c r="D42" s="15" t="s">
         <v>163</v>
       </c>
-      <c r="E42" s="20">
-        <v>8</v>
-      </c>
-      <c r="F42" s="20" t="s">
+      <c r="E42" s="22">
+        <v>8</v>
+      </c>
+      <c r="F42" s="22" t="s">
         <v>164</v>
       </c>
-      <c r="G42" s="20" t="s">
+      <c r="G42" s="22" t="s">
         <v>164</v>
       </c>
-      <c r="H42" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I42" s="13" t="s">
+      <c r="H42" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I42" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="43" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="22">
+    <row r="43" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="24">
         <v>42</v>
       </c>
-      <c r="B43" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C43" s="23" t="s">
+      <c r="B43" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C43" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="D43" s="23" t="s">
+      <c r="D43" s="25" t="s">
         <v>165</v>
       </c>
-      <c r="E43" s="22">
-        <v>8</v>
-      </c>
-      <c r="F43" s="22" t="s">
+      <c r="E43" s="24">
+        <v>8</v>
+      </c>
+      <c r="F43" s="24" t="s">
         <v>166</v>
       </c>
-      <c r="G43" s="22" t="s">
+      <c r="G43" s="24" t="s">
         <v>166</v>
       </c>
-      <c r="H43" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I43" s="13" t="s">
+      <c r="H43" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I43" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="44" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="20">
+    <row r="44" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="22">
         <v>43</v>
       </c>
-      <c r="B44" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C44" s="13" t="s">
+      <c r="B44" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C44" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="D44" s="13" t="s">
+      <c r="D44" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="E44" s="20">
-        <v>8</v>
-      </c>
-      <c r="F44" s="20" t="s">
+      <c r="E44" s="22">
+        <v>8</v>
+      </c>
+      <c r="F44" s="22" t="s">
         <v>168</v>
       </c>
-      <c r="G44" s="20" t="s">
+      <c r="G44" s="22" t="s">
         <v>168</v>
       </c>
-      <c r="H44" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I44" s="13" t="s">
+      <c r="H44" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I44" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="45" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="22">
+    <row r="45" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="24">
         <v>44</v>
       </c>
-      <c r="B45" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C45" s="23" t="s">
+      <c r="B45" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C45" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="D45" s="23" t="s">
+      <c r="D45" s="25" t="s">
         <v>169</v>
       </c>
-      <c r="E45" s="22">
-        <v>8</v>
-      </c>
-      <c r="F45" s="22" t="s">
+      <c r="E45" s="24">
+        <v>8</v>
+      </c>
+      <c r="F45" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="G45" s="22" t="s">
+      <c r="G45" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="H45" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I45" s="13" t="s">
+      <c r="H45" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I45" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="46" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="20">
+    <row r="46" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="22">
         <v>45</v>
       </c>
-      <c r="B46" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C46" s="13" t="s">
+      <c r="B46" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C46" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="D46" s="13" t="s">
+      <c r="D46" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="E46" s="20">
-        <v>8</v>
-      </c>
-      <c r="F46" s="20" t="s">
+      <c r="E46" s="22">
+        <v>8</v>
+      </c>
+      <c r="F46" s="22" t="s">
         <v>172</v>
       </c>
-      <c r="G46" s="20" t="s">
+      <c r="G46" s="22" t="s">
         <v>172</v>
       </c>
-      <c r="H46" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I46" s="13" t="s">
+      <c r="H46" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I46" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="47" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="22">
+    <row r="47" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="24">
         <v>46</v>
       </c>
-      <c r="B47" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C47" s="23" t="s">
+      <c r="B47" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C47" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="D47" s="23" t="s">
+      <c r="D47" s="25" t="s">
         <v>173</v>
       </c>
-      <c r="E47" s="22">
-        <v>8</v>
-      </c>
-      <c r="F47" s="22" t="s">
+      <c r="E47" s="24">
+        <v>8</v>
+      </c>
+      <c r="F47" s="24" t="s">
         <v>174</v>
       </c>
-      <c r="G47" s="22" t="s">
+      <c r="G47" s="24" t="s">
         <v>174</v>
       </c>
-      <c r="H47" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I47" s="13" t="s">
+      <c r="H47" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I47" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="48" spans="1:9" s="13" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="17">
+    <row r="48" ht="36" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="19">
         <v>47</v>
       </c>
-      <c r="B48" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="C48" s="18" t="s">
+      <c r="B48" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="C48" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="D48" s="19" t="s">
+      <c r="D48" s="21" t="s">
         <v>175</v>
       </c>
-      <c r="E48" s="17">
+      <c r="E48" s="19">
         <v>16</v>
       </c>
-      <c r="F48" s="17" t="s">
+      <c r="F48" s="19" t="s">
         <v>176</v>
       </c>
-      <c r="G48" s="17" t="s">
+      <c r="G48" s="19" t="s">
         <v>177</v>
       </c>
-      <c r="H48" s="24" t="s">
+      <c r="H48" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="I48" s="13" t="s">
+      <c r="I48" s="15" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="49" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="22">
+    <row r="49" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="24">
         <v>48</v>
       </c>
-      <c r="B49" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C49" s="23" t="s">
+      <c r="B49" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C49" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="D49" s="23" t="s">
+      <c r="D49" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="E49" s="22">
-        <v>8</v>
-      </c>
-      <c r="F49" s="22" t="s">
+      <c r="E49" s="24">
+        <v>8</v>
+      </c>
+      <c r="F49" s="24" t="s">
         <v>179</v>
       </c>
-      <c r="G49" s="22" t="s">
+      <c r="G49" s="24" t="s">
         <v>179</v>
       </c>
-      <c r="H49" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I49" s="13" t="s">
+      <c r="H49" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I49" s="15" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="50" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="20">
-        <v>49</v>
-      </c>
-      <c r="B50" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C50" s="13" t="s">
+    <row r="50" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="22">
+        <v>49</v>
+      </c>
+      <c r="B50" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C50" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="D50" s="13" t="s">
+      <c r="D50" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="E50" s="20">
-        <v>8</v>
-      </c>
-      <c r="F50" s="20" t="s">
+      <c r="E50" s="22">
+        <v>8</v>
+      </c>
+      <c r="F50" s="22" t="s">
         <v>181</v>
       </c>
-      <c r="G50" s="20" t="s">
+      <c r="G50" s="22" t="s">
         <v>181</v>
       </c>
-      <c r="H50" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I50" s="13" t="s">
+      <c r="H50" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I50" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="51" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="22">
+    <row r="51" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="24">
         <v>50</v>
       </c>
-      <c r="B51" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C51" s="23" t="s">
+      <c r="B51" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C51" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="D51" s="23" t="s">
+      <c r="D51" s="25" t="s">
         <v>66</v>
       </c>
-      <c r="E51" s="22">
-        <v>8</v>
-      </c>
-      <c r="F51" s="22" t="s">
+      <c r="E51" s="24">
+        <v>8</v>
+      </c>
+      <c r="F51" s="24" t="s">
         <v>182</v>
       </c>
-      <c r="G51" s="22" t="s">
+      <c r="G51" s="24" t="s">
         <v>182</v>
       </c>
-      <c r="H51" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I51" s="13" t="s">
+      <c r="H51" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I51" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="52" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="20">
+    <row r="52" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="22">
         <v>51</v>
       </c>
-      <c r="B52" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C52" s="13" t="s">
+      <c r="B52" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C52" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="D52" s="13" t="s">
+      <c r="D52" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="E52" s="20">
-        <v>8</v>
-      </c>
-      <c r="F52" s="20" t="s">
+      <c r="E52" s="22">
+        <v>8</v>
+      </c>
+      <c r="F52" s="22" t="s">
         <v>183</v>
       </c>
-      <c r="G52" s="20" t="s">
+      <c r="G52" s="22" t="s">
         <v>183</v>
       </c>
-      <c r="H52" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I52" s="13" t="s">
+      <c r="H52" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I52" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="53" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="22">
+    <row r="53" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="24">
         <v>52</v>
       </c>
-      <c r="B53" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C53" s="23" t="s">
+      <c r="B53" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C53" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="D53" s="23" t="s">
+      <c r="D53" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="E53" s="22">
-        <v>8</v>
-      </c>
-      <c r="F53" s="22" t="s">
+      <c r="E53" s="24">
+        <v>8</v>
+      </c>
+      <c r="F53" s="24" t="s">
         <v>184</v>
       </c>
-      <c r="G53" s="22" t="s">
+      <c r="G53" s="24" t="s">
         <v>184</v>
       </c>
-      <c r="H53" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I53" s="13" t="s">
+      <c r="H53" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I53" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="54" spans="1:9" s="13" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="17">
+    <row r="54" ht="36" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="19">
         <v>53</v>
       </c>
-      <c r="B54" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="C54" s="18" t="s">
+      <c r="B54" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="C54" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="D54" s="19" t="s">
+      <c r="D54" s="21" t="s">
         <v>185</v>
       </c>
-      <c r="E54" s="17">
-        <v>8</v>
-      </c>
-      <c r="F54" s="17" t="s">
+      <c r="E54" s="19">
+        <v>8</v>
+      </c>
+      <c r="F54" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="G54" s="17" t="s">
+      <c r="G54" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="H54" s="24" t="s">
+      <c r="H54" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="I54" s="13" t="s">
+      <c r="I54" s="15" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="55" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="22">
+    <row r="55" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="24">
         <v>54</v>
       </c>
-      <c r="B55" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C55" s="23" t="s">
+      <c r="B55" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C55" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="D55" s="23" t="s">
+      <c r="D55" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="E55" s="22">
-        <v>8</v>
-      </c>
-      <c r="F55" s="22" t="s">
+      <c r="E55" s="24">
+        <v>8</v>
+      </c>
+      <c r="F55" s="24" t="s">
         <v>188</v>
       </c>
-      <c r="G55" s="22" t="s">
+      <c r="G55" s="24" t="s">
         <v>188</v>
       </c>
-      <c r="H55" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I55" s="13" t="s">
+      <c r="H55" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I55" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="56" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="20">
+    <row r="56" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="22">
         <v>55</v>
       </c>
-      <c r="B56" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C56" s="13" t="s">
+      <c r="B56" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C56" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="D56" s="13" t="s">
+      <c r="D56" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="E56" s="20">
-        <v>8</v>
-      </c>
-      <c r="F56" s="20" t="s">
+      <c r="E56" s="22">
+        <v>8</v>
+      </c>
+      <c r="F56" s="22" t="s">
         <v>189</v>
       </c>
-      <c r="G56" s="20" t="s">
+      <c r="G56" s="22" t="s">
         <v>189</v>
       </c>
-      <c r="H56" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I56" s="13" t="s">
+      <c r="H56" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I56" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="57" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="22">
+    <row r="57" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="24">
         <v>56</v>
       </c>
-      <c r="B57" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C57" s="23" t="s">
+      <c r="B57" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C57" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="D57" s="23" t="s">
+      <c r="D57" s="25" t="s">
         <v>190</v>
       </c>
-      <c r="E57" s="22">
-        <v>8</v>
-      </c>
-      <c r="F57" s="22" t="s">
+      <c r="E57" s="24">
+        <v>8</v>
+      </c>
+      <c r="F57" s="24" t="s">
         <v>191</v>
       </c>
-      <c r="G57" s="22" t="s">
+      <c r="G57" s="24" t="s">
         <v>191</v>
       </c>
-      <c r="H57" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I57" s="13" t="s">
+      <c r="H57" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I57" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="58" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="20">
+    <row r="58" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="22">
         <v>57</v>
       </c>
-      <c r="B58" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C58" s="13" t="s">
+      <c r="B58" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C58" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="D58" s="13" t="s">
+      <c r="D58" s="15" t="s">
         <v>192</v>
       </c>
-      <c r="E58" s="20">
-        <v>8</v>
-      </c>
-      <c r="F58" s="20" t="s">
+      <c r="E58" s="22">
+        <v>8</v>
+      </c>
+      <c r="F58" s="22" t="s">
         <v>193</v>
       </c>
-      <c r="G58" s="20" t="s">
+      <c r="G58" s="22" t="s">
         <v>193</v>
       </c>
-      <c r="H58" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I58" s="13" t="s">
+      <c r="H58" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I58" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="59" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="22">
+    <row r="59" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="24">
         <v>58</v>
       </c>
-      <c r="B59" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C59" s="23" t="s">
+      <c r="B59" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C59" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="D59" s="23" t="s">
+      <c r="D59" s="25" t="s">
         <v>194</v>
       </c>
-      <c r="E59" s="22">
-        <v>8</v>
-      </c>
-      <c r="F59" s="22" t="s">
+      <c r="E59" s="24">
+        <v>8</v>
+      </c>
+      <c r="F59" s="24" t="s">
         <v>195</v>
       </c>
-      <c r="G59" s="22" t="s">
+      <c r="G59" s="24" t="s">
         <v>195</v>
       </c>
-      <c r="H59" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I59" s="13" t="s">
+      <c r="H59" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I59" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="60" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="20">
+    <row r="60" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="22">
         <v>59</v>
       </c>
-      <c r="B60" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C60" s="13" t="s">
+      <c r="B60" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C60" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="D60" s="13" t="s">
+      <c r="D60" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="E60" s="20">
-        <v>8</v>
-      </c>
-      <c r="F60" s="20" t="s">
+      <c r="E60" s="22">
+        <v>8</v>
+      </c>
+      <c r="F60" s="22" t="s">
         <v>196</v>
       </c>
-      <c r="G60" s="20" t="s">
+      <c r="G60" s="22" t="s">
         <v>196</v>
       </c>
-      <c r="H60" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I60" s="13" t="s">
+      <c r="H60" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I60" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="61" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="22">
+    <row r="61" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="24">
         <v>60</v>
       </c>
-      <c r="B61" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C61" s="23" t="s">
+      <c r="B61" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C61" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="D61" s="23" t="s">
+      <c r="D61" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="E61" s="22">
-        <v>8</v>
-      </c>
-      <c r="F61" s="22" t="s">
+      <c r="E61" s="24">
+        <v>8</v>
+      </c>
+      <c r="F61" s="24" t="s">
         <v>197</v>
       </c>
-      <c r="G61" s="22" t="s">
+      <c r="G61" s="24" t="s">
         <v>197</v>
       </c>
-      <c r="H61" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I61" s="13" t="s">
+      <c r="H61" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I61" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="62" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="20">
+    <row r="62" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="22">
         <v>61</v>
       </c>
-      <c r="B62" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C62" s="13" t="s">
+      <c r="B62" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C62" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="D62" s="13" t="s">
+      <c r="D62" s="15" t="s">
         <v>198</v>
       </c>
-      <c r="E62" s="20">
-        <v>8</v>
-      </c>
-      <c r="F62" s="20" t="s">
+      <c r="E62" s="22">
+        <v>8</v>
+      </c>
+      <c r="F62" s="22" t="s">
         <v>199</v>
       </c>
-      <c r="G62" s="20" t="s">
+      <c r="G62" s="22" t="s">
         <v>199</v>
       </c>
-      <c r="H62" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I62" s="13" t="s">
+      <c r="H62" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I62" s="15" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="63" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="22">
+    <row r="63" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="24">
         <v>62</v>
       </c>
-      <c r="B63" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C63" s="23" t="s">
+      <c r="B63" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C63" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="D63" s="23" t="s">
+      <c r="D63" s="25" t="s">
         <v>201</v>
       </c>
-      <c r="E63" s="22">
-        <v>8</v>
-      </c>
-      <c r="F63" s="22" t="s">
+      <c r="E63" s="24">
+        <v>8</v>
+      </c>
+      <c r="F63" s="24" t="s">
         <v>202</v>
       </c>
-      <c r="G63" s="22" t="s">
+      <c r="G63" s="24" t="s">
         <v>202</v>
       </c>
-      <c r="H63" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I63" s="13" t="s">
+      <c r="H63" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I63" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="64" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="20">
+    <row r="64" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="22">
         <v>63</v>
       </c>
-      <c r="B64" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C64" s="13" t="s">
+      <c r="B64" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C64" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="D64" s="13" t="s">
+      <c r="D64" s="15" t="s">
         <v>203</v>
       </c>
-      <c r="E64" s="20">
-        <v>8</v>
-      </c>
-      <c r="F64" s="20" t="s">
+      <c r="E64" s="22">
+        <v>8</v>
+      </c>
+      <c r="F64" s="22" t="s">
         <v>204</v>
       </c>
-      <c r="G64" s="20" t="s">
+      <c r="G64" s="22" t="s">
         <v>204</v>
       </c>
-      <c r="H64" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I64" s="13" t="s">
+      <c r="H64" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I64" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="65" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="22">
+    <row r="65" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="24">
         <v>64</v>
       </c>
-      <c r="B65" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C65" s="23" t="s">
+      <c r="B65" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C65" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="D65" s="23" t="s">
+      <c r="D65" s="25" t="s">
         <v>205</v>
       </c>
-      <c r="E65" s="22">
-        <v>8</v>
-      </c>
-      <c r="F65" s="22" t="s">
+      <c r="E65" s="24">
+        <v>8</v>
+      </c>
+      <c r="F65" s="24" t="s">
         <v>206</v>
       </c>
-      <c r="G65" s="22" t="s">
+      <c r="G65" s="24" t="s">
         <v>206</v>
       </c>
-      <c r="H65" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I65" s="13" t="s">
+      <c r="H65" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I65" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="66" spans="1:9" s="13" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="17">
+    <row r="66" ht="36" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="19">
         <v>65</v>
       </c>
-      <c r="B66" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="C66" s="18" t="s">
+      <c r="B66" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="C66" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="D66" s="19" t="s">
+      <c r="D66" s="21" t="s">
         <v>207</v>
       </c>
-      <c r="E66" s="17">
+      <c r="E66" s="19">
         <v>24</v>
       </c>
-      <c r="F66" s="17" t="s">
+      <c r="F66" s="19" t="s">
         <v>208</v>
       </c>
-      <c r="G66" s="17" t="s">
+      <c r="G66" s="19" t="s">
         <v>209</v>
       </c>
-      <c r="H66" s="24" t="s">
+      <c r="H66" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="I66" s="13" t="s">
+      <c r="I66" s="15" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="67" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="22">
+    <row r="67" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="24">
         <v>66</v>
       </c>
-      <c r="B67" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C67" s="23" t="s">
+      <c r="B67" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C67" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="D67" s="23" t="s">
+      <c r="D67" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="E67" s="22">
-        <v>8</v>
-      </c>
-      <c r="F67" s="22" t="s">
+      <c r="E67" s="24">
+        <v>8</v>
+      </c>
+      <c r="F67" s="24" t="s">
         <v>211</v>
       </c>
-      <c r="G67" s="22" t="s">
+      <c r="G67" s="24" t="s">
         <v>211</v>
       </c>
-      <c r="H67" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I67" s="13" t="s">
+      <c r="H67" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I67" s="15" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="68" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="20">
+    <row r="68" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="22">
         <v>67</v>
       </c>
-      <c r="B68" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C68" s="13" t="s">
+      <c r="B68" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C68" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="D68" s="13" t="s">
+      <c r="D68" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="E68" s="20">
-        <v>8</v>
-      </c>
-      <c r="F68" s="20" t="s">
+      <c r="E68" s="22">
+        <v>8</v>
+      </c>
+      <c r="F68" s="22" t="s">
         <v>213</v>
       </c>
-      <c r="G68" s="20" t="s">
+      <c r="G68" s="22" t="s">
         <v>213</v>
       </c>
-      <c r="H68" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I68" s="13" t="s">
+      <c r="H68" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I68" s="15" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="69" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="22">
+    <row r="69" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="24">
         <v>68</v>
       </c>
-      <c r="B69" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C69" s="23" t="s">
+      <c r="B69" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C69" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="D69" s="23" t="s">
+      <c r="D69" s="25" t="s">
         <v>190</v>
       </c>
-      <c r="E69" s="22">
-        <v>8</v>
-      </c>
-      <c r="F69" s="22" t="s">
+      <c r="E69" s="24">
+        <v>8</v>
+      </c>
+      <c r="F69" s="24" t="s">
         <v>215</v>
       </c>
-      <c r="G69" s="22" t="s">
+      <c r="G69" s="24" t="s">
         <v>215</v>
       </c>
-      <c r="H69" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I69" s="13" t="s">
+      <c r="H69" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I69" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="70" spans="1:9" s="13" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="17">
+    <row r="70" ht="36" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="19">
         <v>69</v>
       </c>
-      <c r="B70" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="C70" s="18" t="s">
+      <c r="B70" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="C70" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="D70" s="19" t="s">
+      <c r="D70" s="21" t="s">
         <v>216</v>
       </c>
-      <c r="E70" s="17">
+      <c r="E70" s="19">
         <v>4</v>
       </c>
-      <c r="F70" s="17" t="s">
+      <c r="F70" s="19" t="s">
         <v>217</v>
       </c>
-      <c r="G70" s="17" t="s">
+      <c r="G70" s="19" t="s">
         <v>217</v>
       </c>
-      <c r="H70" s="24" t="s">
+      <c r="H70" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="I70" s="13" t="s">
+      <c r="I70" s="15" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="71" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="22">
+    <row r="71" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="24">
         <v>70</v>
       </c>
-      <c r="B71" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C71" s="23" t="s">
+      <c r="B71" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C71" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="D71" s="23" t="s">
+      <c r="D71" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="E71" s="22">
-        <v>8</v>
-      </c>
-      <c r="F71" s="22" t="s">
+      <c r="E71" s="24">
+        <v>8</v>
+      </c>
+      <c r="F71" s="24" t="s">
         <v>218</v>
       </c>
-      <c r="G71" s="22" t="s">
+      <c r="G71" s="24" t="s">
         <v>218</v>
       </c>
-      <c r="H71" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I71" s="13" t="s">
+      <c r="H71" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I71" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="72" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="20">
+    <row r="72" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="22">
         <v>71</v>
       </c>
-      <c r="B72" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C72" s="13" t="s">
+      <c r="B72" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C72" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="D72" s="13" t="s">
+      <c r="D72" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="E72" s="20">
-        <v>8</v>
-      </c>
-      <c r="F72" s="20" t="s">
+      <c r="E72" s="22">
+        <v>8</v>
+      </c>
+      <c r="F72" s="22" t="s">
         <v>219</v>
       </c>
-      <c r="G72" s="20" t="s">
+      <c r="G72" s="22" t="s">
         <v>219</v>
       </c>
-      <c r="H72" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I72" s="13" t="s">
+      <c r="H72" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I72" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="73" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="22">
+    <row r="73" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="24">
         <v>72</v>
       </c>
-      <c r="B73" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C73" s="23" t="s">
+      <c r="B73" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C73" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="D73" s="23" t="s">
+      <c r="D73" s="25" t="s">
         <v>190</v>
       </c>
-      <c r="E73" s="22">
-        <v>8</v>
-      </c>
-      <c r="F73" s="22" t="s">
+      <c r="E73" s="24">
+        <v>8</v>
+      </c>
+      <c r="F73" s="24" t="s">
         <v>220</v>
       </c>
-      <c r="G73" s="22" t="s">
+      <c r="G73" s="24" t="s">
         <v>220</v>
       </c>
-      <c r="H73" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I73" s="13" t="s">
+      <c r="H73" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I73" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="74" spans="1:9" s="13" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="17">
+    <row r="74" ht="36" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="19">
         <v>73</v>
       </c>
-      <c r="B74" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="C74" s="18" t="s">
+      <c r="B74" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="C74" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="D74" s="19" t="s">
+      <c r="D74" s="21" t="s">
         <v>221</v>
       </c>
-      <c r="E74" s="17">
+      <c r="E74" s="19">
         <v>4</v>
       </c>
-      <c r="F74" s="17" t="s">
+      <c r="F74" s="19" t="s">
         <v>222</v>
       </c>
-      <c r="G74" s="17" t="s">
+      <c r="G74" s="19" t="s">
         <v>222</v>
       </c>
-      <c r="H74" s="24" t="s">
+      <c r="H74" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="I74" s="13" t="s">
+      <c r="I74" s="15" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="75" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="22">
+    <row r="75" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="24">
         <v>74</v>
       </c>
-      <c r="B75" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C75" s="23" t="s">
+      <c r="B75" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C75" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="D75" s="23" t="s">
+      <c r="D75" s="25" t="s">
         <v>223</v>
       </c>
-      <c r="E75" s="22">
-        <v>8</v>
-      </c>
-      <c r="F75" s="22" t="s">
+      <c r="E75" s="24">
+        <v>8</v>
+      </c>
+      <c r="F75" s="24" t="s">
         <v>224</v>
       </c>
-      <c r="G75" s="22" t="s">
+      <c r="G75" s="24" t="s">
         <v>224</v>
       </c>
-      <c r="H75" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I75" s="13" t="s">
+      <c r="H75" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I75" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="76" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="20">
+    <row r="76" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="22">
         <v>75</v>
       </c>
-      <c r="B76" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C76" s="13" t="s">
+      <c r="B76" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C76" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="D76" s="13" t="s">
+      <c r="D76" s="15" t="s">
         <v>225</v>
       </c>
-      <c r="E76" s="20">
-        <v>8</v>
-      </c>
-      <c r="F76" s="20" t="s">
+      <c r="E76" s="22">
+        <v>8</v>
+      </c>
+      <c r="F76" s="22" t="s">
         <v>226</v>
       </c>
-      <c r="G76" s="20" t="s">
+      <c r="G76" s="22" t="s">
         <v>226</v>
       </c>
-      <c r="H76" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I76" s="13" t="s">
+      <c r="H76" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I76" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="77" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="22">
+    <row r="77" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="24">
         <v>76</v>
       </c>
-      <c r="B77" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C77" s="23" t="s">
+      <c r="B77" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C77" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="D77" s="23" t="s">
+      <c r="D77" s="25" t="s">
         <v>227</v>
       </c>
-      <c r="E77" s="22">
-        <v>8</v>
-      </c>
-      <c r="F77" s="22" t="s">
+      <c r="E77" s="24">
+        <v>8</v>
+      </c>
+      <c r="F77" s="24" t="s">
         <v>228</v>
       </c>
-      <c r="G77" s="22" t="s">
+      <c r="G77" s="24" t="s">
         <v>228</v>
       </c>
-      <c r="H77" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I77" s="13" t="s">
+      <c r="H77" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I77" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="78" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="20">
+    <row r="78" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="22">
         <v>77</v>
       </c>
-      <c r="B78" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C78" s="13" t="s">
+      <c r="B78" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C78" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="D78" s="13" t="s">
+      <c r="D78" s="15" t="s">
         <v>229</v>
       </c>
-      <c r="E78" s="20">
-        <v>8</v>
-      </c>
-      <c r="F78" s="20" t="s">
+      <c r="E78" s="22">
+        <v>8</v>
+      </c>
+      <c r="F78" s="22" t="s">
         <v>230</v>
       </c>
-      <c r="G78" s="20" t="s">
+      <c r="G78" s="22" t="s">
         <v>230</v>
       </c>
-      <c r="H78" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I78" s="13" t="s">
+      <c r="H78" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I78" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="79" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="22">
+    <row r="79" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="24">
         <v>78</v>
       </c>
-      <c r="B79" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C79" s="23" t="s">
+      <c r="B79" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C79" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="D79" s="23" t="s">
+      <c r="D79" s="25" t="s">
         <v>231</v>
       </c>
-      <c r="E79" s="22">
-        <v>8</v>
-      </c>
-      <c r="F79" s="22" t="s">
+      <c r="E79" s="24">
+        <v>8</v>
+      </c>
+      <c r="F79" s="24" t="s">
         <v>232</v>
       </c>
-      <c r="G79" s="22" t="s">
+      <c r="G79" s="24" t="s">
         <v>232</v>
       </c>
-      <c r="H79" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I79" s="13" t="s">
+      <c r="H79" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I79" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="80" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="20">
+    <row r="80" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="22">
         <v>79</v>
       </c>
-      <c r="B80" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C80" s="13" t="s">
+      <c r="B80" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C80" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="D80" s="13" t="s">
+      <c r="D80" s="15" t="s">
         <v>233</v>
       </c>
-      <c r="E80" s="20">
-        <v>8</v>
-      </c>
-      <c r="F80" s="20" t="s">
+      <c r="E80" s="22">
+        <v>8</v>
+      </c>
+      <c r="F80" s="22" t="s">
         <v>234</v>
       </c>
-      <c r="G80" s="20" t="s">
+      <c r="G80" s="22" t="s">
         <v>234</v>
       </c>
-      <c r="H80" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I80" s="13" t="s">
+      <c r="H80" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I80" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="81" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="22">
+    <row r="81" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="24">
         <v>80</v>
       </c>
-      <c r="B81" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C81" s="23" t="s">
+      <c r="B81" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C81" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="D81" s="23" t="s">
+      <c r="D81" s="25" t="s">
         <v>235</v>
       </c>
-      <c r="E81" s="22">
-        <v>8</v>
-      </c>
-      <c r="F81" s="22" t="s">
+      <c r="E81" s="24">
+        <v>8</v>
+      </c>
+      <c r="F81" s="24" t="s">
         <v>236</v>
       </c>
-      <c r="G81" s="22" t="s">
+      <c r="G81" s="24" t="s">
         <v>236</v>
       </c>
-      <c r="H81" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I81" s="13" t="s">
+      <c r="H81" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I81" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="82" spans="1:9" s="13" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="17">
+    <row r="82" ht="36" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="19">
         <v>81</v>
       </c>
-      <c r="B82" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="C82" s="18" t="s">
+      <c r="B82" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="C82" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="D82" s="19" t="s">
+      <c r="D82" s="21" t="s">
         <v>237</v>
       </c>
-      <c r="E82" s="17">
+      <c r="E82" s="19">
         <v>16</v>
       </c>
-      <c r="F82" s="17" t="s">
+      <c r="F82" s="19" t="s">
         <v>238</v>
       </c>
-      <c r="G82" s="17" t="s">
+      <c r="G82" s="19" t="s">
         <v>239</v>
       </c>
-      <c r="H82" s="24" t="s">
+      <c r="H82" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="I82" s="13" t="s">
+      <c r="I82" s="15" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="83" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="22">
+    <row r="83" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="24">
         <v>82</v>
       </c>
-      <c r="B83" s="23" t="s">
+      <c r="B83" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="C83" s="23" t="s">
+      <c r="C83" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="D83" s="23" t="s">
+      <c r="D83" s="25" t="s">
         <v>240</v>
       </c>
-      <c r="E83" s="22">
-        <v>8</v>
-      </c>
-      <c r="F83" s="22" t="s">
+      <c r="E83" s="24">
+        <v>8</v>
+      </c>
+      <c r="F83" s="24" t="s">
         <v>241</v>
       </c>
-      <c r="G83" s="22" t="s">
+      <c r="G83" s="24" t="s">
         <v>241</v>
       </c>
-      <c r="H83" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I83" s="13" t="s">
+      <c r="H83" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I83" s="15" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="84" spans="1:9" s="13" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="20">
+    <row r="84" ht="28" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A84" s="22">
         <v>83</v>
       </c>
-      <c r="B84" s="13" t="s">
+      <c r="B84" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="C84" s="13" t="s">
+      <c r="C84" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="D84" s="13" t="s">
+      <c r="D84" s="15" t="s">
         <v>243</v>
       </c>
-      <c r="E84" s="20">
-        <v>8</v>
-      </c>
-      <c r="F84" s="20" t="s">
+      <c r="E84" s="22">
+        <v>8</v>
+      </c>
+      <c r="F84" s="22" t="s">
         <v>244</v>
       </c>
-      <c r="G84" s="20" t="s">
+      <c r="G84" s="22" t="s">
         <v>244</v>
       </c>
-      <c r="H84" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="I84" s="13" t="s">
+      <c r="H84" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I84" s="15" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="85" spans="1:9" s="13" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="17">
+    <row r="85" ht="36" customHeight="1" spans="1:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A85" s="19">
         <v>84</v>
       </c>
-      <c r="B85" s="18" t="s">
+      <c r="B85" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="C85" s="18" t="s">
+      <c r="C85" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="D85" s="19" t="s">
+      <c r="D85" s="21" t="s">
         <v>246</v>
       </c>
-      <c r="E85" s="17">
+      <c r="E85" s="19">
         <v>4</v>
       </c>
-      <c r="F85" s="17" t="s">
+      <c r="F85" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="G85" s="17" t="s">
+      <c r="G85" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="H85" s="24" t="s">
+      <c r="H85" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="I85" s="13" t="s">
+      <c r="I85" s="15" t="s">
         <v>247</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I85" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
-  <dataValidations count="1">
-    <dataValidation type="list" sqref="H2:H85" xr:uid="{00000000-0002-0000-0100-000000000000}">
+  <autoFilter ref="A1:I85"/>
+  <dataValidations count="2">
+    <dataValidation type="list" sqref="H10:H85">
+      <formula1>"Completed,In Progress,Planned,Buffer,Blocked"</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="H2:H85">
       <formula1>"Completed,In Progress,Planned,Buffer,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A38"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="204.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" s="25" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
+    <row r="1" spans="1:1" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="27" t="s">
         <v>248</v>
       </c>
     </row>
@@ -4370,8 +4346,8 @@
         <v>249</v>
       </c>
     </row>
-    <row r="3" spans="1:1" s="26" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="27" t="s">
+    <row r="3" spans="1:1" s="28" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="29" t="s">
         <v>250</v>
       </c>
     </row>
@@ -4395,8 +4371,8 @@
         <v>249</v>
       </c>
     </row>
-    <row r="8" spans="1:1" s="26" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="27" t="s">
+    <row r="8" spans="1:1" s="28" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="29" t="s">
         <v>254</v>
       </c>
     </row>
@@ -4425,8 +4401,8 @@
         <v>249</v>
       </c>
     </row>
-    <row r="14" spans="1:1" s="26" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="27" t="s">
+    <row r="14" spans="1:1" s="28" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="29" t="s">
         <v>259</v>
       </c>
     </row>
@@ -4455,8 +4431,8 @@
         <v>249</v>
       </c>
     </row>
-    <row r="20" spans="1:1" s="26" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="27" t="s">
+    <row r="20" spans="1:1" s="28" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="29" t="s">
         <v>264</v>
       </c>
     </row>
@@ -4485,8 +4461,8 @@
         <v>249</v>
       </c>
     </row>
-    <row r="26" spans="1:1" s="26" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="27" t="s">
+    <row r="26" spans="1:1" s="28" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="29" t="s">
         <v>269</v>
       </c>
     </row>
@@ -4520,8 +4496,8 @@
         <v>249</v>
       </c>
     </row>
-    <row r="33" spans="1:1" s="26" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A33" s="27" t="s">
+    <row r="33" spans="1:1" s="28" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="29" t="s">
         <v>275</v>
       </c>
     </row>
@@ -4552,6 +4528,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>